<commit_message>
Complete verified address data (32/32) and final label outputs
- 全32事業所の郵便番号・住所・正式名称を介護サービス情報公表システム、
  自治体公式サイト、法人公式サイトで確認して addresses.json に収録
- labels.pdf（11ページ）と 送付先確認一覧.xlsx を再生成
- README を追加

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0111t2PWMmaodzorhMY5DBqq
</commit_message>
<xml_diff>
--- a/mailing-labels/送付先確認一覧.xlsx
+++ b/mailing-labels/送付先確認一覧.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1363,472 +1363,900 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所 ばんどう</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所ばんどう</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>合同会社ばんどう</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>306-0052</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>茨城県古河市大山498-4</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>0280-48-3486</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>住所・電話は公表システム法人情報欄＋古河市公式一覧(2026/7/1)で一致。ただし居宅介護支援の単独公表ページが現在閲覧不可。運営状況を電話確認推奨。</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_001_kihon=true&amp;JigyosyoCd=0870401239-00&amp;ServiceCd=110
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所 ファミリー</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所ファミリー</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>株式会社アイ・コーポレーション</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>306-0002</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市三杉町2-10-8</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>0280-31-1330</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>正式名称はスペースなし。法人本店（静町）とは別住所。</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870401502-00&amp;ServiceCd=430
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>イースケア居宅介護支援事業所</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>イースケア居宅介護支援事業所</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>合同会社嘉邦</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>306-0041</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市鴻巣642番地3</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>0280-23-3853</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>公表システム・古河市公式一覧で一致。</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870401692-00&amp;ServiceCd=430
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援センター きずな</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援センターきずな</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>合同会社Lien de famille</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>306-0025</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市原町9-53 コンフォート古河401</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>0280-23-5993</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>正式名称はスペースなし。法人本店（けやき平）とは別住所。マンション名・部屋番号必須。</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870401809-00&amp;ServiceCd=430
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所 愛和苑</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>居宅介護支援事業所 愛和苑</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>社会福祉法人愛和会</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>306-0221</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市駒羽根320-1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>0280-93-0234</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>特養愛和苑併設・電話共通。法人公式サイトでも確認。</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870400546-00&amp;ServiceCd=430
+http://www.ai-wa-kai.com/aiwaen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>つぐみ居宅介護支援事業所総和</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>つぐみ居宅介護支援事業所総和</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>合同会社緒心</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>306-0233</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市西牛谷411-15 セントラルアパートメント202</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>0280-33-6440</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>別法人(合同会社Rフィールド)の「つぐみ居宅介護支援事業所」(南間中橋)とは別。法人本店（下大野）とは別住所。</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870401957-00&amp;ServiceCd=430
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>介護保険支援センター青嵐荘(総和)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>介護保険支援センター青嵐荘（総和）</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>社会福祉法人芳香会</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>306-0233</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市西牛谷852-4 タウンハウスMITA 105号室</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>0280-98-0030</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>法人公式サイト・古河市公式一覧で一致。古い住所（東牛谷456-6）が地図サイトに残っているが現行は西牛谷852-4。</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.houkoukai.or.jp/jigyou/consultation/index.php?p=kaigohoken-seiran
+https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>古河市地域包括支援センター総和</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>古河市地域包括支援センター総和</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>306-0201</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>茨城県古河市上大野1889-1 特別養護老人ホーム希望の森内</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>0280-23-5661</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>委託先は社会福祉法人愛和会。愛称「高齢者サポートセンター総和」。茨城県一覧(R8.4.1)・古河市公式で一致。</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/5/1685.html
+https://www.pref.ibaraki.jp/hokenfukushi/chofuku/shichoson/kaigo/hokatsu/documents/houkatusentar8.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>総和中央病院 居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>総和中央病院 居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>医療法人仁寿会</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>306-0221</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市駒羽根825-1</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>0280-91-1256</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>公表システム・古河市公式一覧で一致。</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0874300031-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+    <row r="27">
+      <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>あずみ苑古河</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>あずみ苑古河</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>株式会社アズ・ライフケア</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>306-0126</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市諸川1393-2</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>0280-75-1433</t>
         </is>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>居宅介護支援事業所の登録名は「あずみ苑古河」のみ（接尾なし）。デイ・ショートと同一住所・電話。公式サイトでも確認。</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870400561-00&amp;ServiceCd=430
 https://www.azumien.jp/search/koga/</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+    <row r="28">
+      <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>けやきの舎居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>けやきの舎居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>社会医療法人友志会</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>306-0125</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市仁連601</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>0280-77-3335</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>公表システム・古河市公式一覧で一致。</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870400637-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
+    <row r="29">
+      <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>居宅介護支援事業所 きぼう</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>居宅介護支援事業所 きぼう</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>株式会社きぼう</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>306-0126</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>茨城県古河市諸川1307-25</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>0280-75-0707</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H29" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>古河市公式一覧(2026/7/1更新)で名称・住所・電話一致。ただし公表システムの詳細ページが現在閲覧不可（未公表/取下げの可能性）。郵便番号306-0126は諸川の郵便番号として整合。運営状況を電話確認推奨。</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html
 https://r-guide.jp/care_office/79076/</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+    <row r="30">
+      <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>ケアプランセンター四季の郷</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>ケアプランセンター 四季の郷</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>社会福祉法人さしま福祉会</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>306-0107</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市東間中橋198</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>0280-33-3311</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="H30" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>登録名は「ケアプランセンター 四季の郷」（スペースあり）。特養四季の郷と同一建物。</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0870401247-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+    <row r="31">
+      <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>みどりの里指定居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>みどりの里指定居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>社会福祉法人三和みつなみ会</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>306-0112</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市東山田4796-2</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>0280-78-1123</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H31" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>特養・ケアハウスみどりの里と同一住所。</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0874300304-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="32">
+      <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>居宅介護支援センターみどりの丘</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>居宅介護支援センターみどりの丘</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>社会福祉法人三和みつなみ会</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>306-0101</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市尾崎3373</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>0280-75-0770</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>デイサービスセンターみどりの丘と同一敷地。</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0874301021-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>ライフサポートふくろう居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>ライフサポートふくろう居宅介護支援事業所</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>有限会社魁星舎</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>306-0101</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>茨城県古河市尾崎2630番地13</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>0280-75-1335</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>公表システムで住所・電話一致。</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>https://www.kaigokensaku.mhlw.go.jp/08/index.php?action_kouhyou_detail_023_kihon=true&amp;JigyosyoCd=0874301039-00&amp;ServiceCd=430
 https://www.city.ibaraki-koga.lg.jp/soshiki/koureikaigo/ippan/4/12356.html</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>24事業所</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="I27" s="2" t="n"/>
-      <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>32事業所</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>